<commit_message>
new updates on the formatting of the app
</commit_message>
<xml_diff>
--- a/Raw_eGRID_EF_2025.xlsx
+++ b/Raw_eGRID_EF_2025.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="24" documentId="13_ncr:1_{FB31CA3F-A5DC-4EA1-BF05-0E89501011C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{730D06CD-9D40-463C-A752-75B88CC144E0}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{684B57A3-FFB1-4E11-B6A1-72CE2EF8511A}"/>
+    <workbookView xWindow="-19812" yWindow="-17388" windowWidth="30936" windowHeight="16776" xr2:uid="{684B57A3-FFB1-4E11-B6A1-72CE2EF8511A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>